<commit_message>
Switch default scenario to BAU and drop stale NDC outputs
- Config: Main_Scenario NDC -> BAU, enable_dsptrn true
- D2: read TRN limits from dedicated TRN_Flow_Limits sheet (keeps Editor
  untouched for manual edits), merge into instructions at apply time
- Remove legacy scenario outputs (NDC, NDC+ELC, NDC_NoRPO) and
  A2_Outputs_Params_otoole/NDC CSVs now that BAU is the active run
- Add parametrization review workflow: AUX_Z_recalc_shares.py,
  D3_load_lac_max_capacity_caps.py, Z_AUX_apply_parametrization_review.py
  and A-O_Parametrization_Review_PWR/Tx md+xlsx outputs
- Add project docs (installation, quickstart, pipeline, configuration,
  country-management, data-reference, auxiliary-tools)
- Refresh BAU outputs and inputs (shares, growth goals, emissions, storage,
  secondary techs editor)
</commit_message>
<xml_diff>
--- a/t1_confection/RateGrowthDemand_RenovabilityGoals.xlsx
+++ b/t1_confection/RateGrowthDemand_RenovabilityGoals.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\relac_tx\t1_confection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{054E976C-9A52-4BBB-8209-C652C7181E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFE571F-4EC0-48B1-94E0-D8AAA1C4227E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{82D8F5DC-00C5-4DE6-8A6C-5F3405DB195A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82D8F5DC-00C5-4DE6-8A6C-5F3405DB195A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -373,12 +373,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -394,7 +400,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -419,6 +425,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -775,7 +790,7 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
@@ -798,7 +813,7 @@
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="10" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -821,7 +836,7 @@
       <c r="D3" s="2">
         <v>16.3</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="11">
         <v>6.3799999999999996E-2</v>
       </c>
       <c r="F3" s="6">
@@ -844,7 +859,7 @@
       <c r="D4" s="2">
         <v>110.7</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="11">
         <v>5.3400000000000003E-2</v>
       </c>
       <c r="F4" s="6">
@@ -867,7 +882,7 @@
       <c r="D5" s="2">
         <v>81.2</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="11">
         <v>3.6900000000000002E-2</v>
       </c>
       <c r="F5" s="6">
@@ -890,7 +905,7 @@
       <c r="D6" s="2">
         <v>11.3</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="11">
         <v>2.06E-2</v>
       </c>
       <c r="F6" s="6">
@@ -913,7 +928,7 @@
       <c r="D7" s="2">
         <v>28.3</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="11">
         <v>4.5600000000000002E-2</v>
       </c>
       <c r="F7" s="6">
@@ -936,7 +951,7 @@
       <c r="D8" s="2">
         <v>7</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="11">
         <v>2.3099999999999999E-2</v>
       </c>
       <c r="F8" s="6">
@@ -959,7 +974,7 @@
       <c r="D9" s="2">
         <v>0.9</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="11">
         <v>3.2300000000000002E-2</v>
       </c>
       <c r="F9" s="6">
@@ -982,7 +997,7 @@
       <c r="D10" s="2">
         <v>8</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="11">
         <v>3.0599999999999999E-2</v>
       </c>
       <c r="F10" s="6">
@@ -1005,7 +1020,7 @@
       <c r="D11" s="2">
         <v>4.5999999999999996</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="11">
         <v>4.5699999999999998E-2</v>
       </c>
       <c r="F11" s="6">
@@ -1028,7 +1043,7 @@
       <c r="D12" s="2">
         <v>11.2</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="11">
         <v>4.87E-2</v>
       </c>
       <c r="F12" s="6">
@@ -1051,7 +1066,7 @@
       <c r="D13" s="2">
         <v>16.3</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="11">
         <v>6.3799999999999996E-2</v>
       </c>
       <c r="F13" s="6">
@@ -1074,7 +1089,7 @@
       <c r="D14" s="2">
         <v>53.2</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="11">
         <v>4.2799999999999998E-2</v>
       </c>
       <c r="F14" s="6">
@@ -1097,7 +1112,7 @@
       <c r="D15" s="2">
         <v>19.3</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="11">
         <v>3.5000000000000003E-2</v>
       </c>
       <c r="F15" s="6">
@@ -1120,7 +1135,7 @@
       <c r="D16" s="2">
         <v>12.2</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="11">
         <v>2.3599999999999999E-2</v>
       </c>
       <c r="F16" s="6">
@@ -1143,7 +1158,7 @@
       <c r="D17" s="2">
         <v>615.79999999999995</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="11">
         <v>2.1899999999999999E-2</v>
       </c>
       <c r="F17" s="6">
@@ -1166,7 +1181,7 @@
       <c r="D18" s="2">
         <v>128.5</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="11">
         <v>8.8000000000000005E-3</v>
       </c>
       <c r="F18" s="6">
@@ -1189,7 +1204,7 @@
       <c r="D19" s="2">
         <v>338.4</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="11">
         <v>0.03</v>
       </c>
       <c r="F19" s="6">
@@ -1212,7 +1227,7 @@
       <c r="D20" s="2">
         <v>12</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="11">
         <v>3.4799999999999998E-2</v>
       </c>
       <c r="F20" s="6">

</xml_diff>